<commit_message>
feat: Add explicit per-step acceptance checkpoints and StepAcceptanceError fuse mechanism
</commit_message>
<xml_diff>
--- a/examples/case_study_corticosteroids_nma/editable_files/office_docs/Master_Research_Database.xlsx
+++ b/examples/case_study_corticosteroids_nma/editable_files/office_docs/Master_Research_Database.xlsx
@@ -2646,7 +2646,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Hydrocortisone + Fludrocortisone</t>
+          <t>Methylprednisolone</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -2659,16 +2659,16 @@
         <v>1</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>0.76</v>
+        <v>0.82</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>1.32</v>
+        <v>1.22</v>
       </c>
     </row>
     <row r="3" ht="20" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Dexamethasone</t>
+          <t>Hydrocortisone</t>
         </is>
       </c>
       <c r="B3" s="2" t="n">
@@ -2681,16 +2681,16 @@
         <v>1</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>0.76</v>
+        <v>0.92</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>1.32</v>
+        <v>1.09</v>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Methylprednisolone</t>
+          <t>Hydrocortisone + Fludrocortisone</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -2703,16 +2703,16 @@
         <v>1</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>0.82</v>
+        <v>0.76</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>1.22</v>
+        <v>1.32</v>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Hydrocortisone</t>
+          <t>Dexamethasone</t>
         </is>
       </c>
       <c r="B5" s="2" t="n">
@@ -2725,10 +2725,10 @@
         <v>1</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>0.92</v>
+        <v>0.76</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>1.09</v>
+        <v>1.32</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">

</xml_diff>

<commit_message>
feat: upgrade literature search and screening workflow with institutional session reuse, full corpus landing, multi-tier provenance deduplication, and two-stage screening ledger
</commit_message>
<xml_diff>
--- a/examples/case_study_corticosteroids_nma/editable_files/office_docs/Master_Research_Database.xlsx
+++ b/examples/case_study_corticosteroids_nma/editable_files/office_docs/Master_Research_Database.xlsx
@@ -2668,7 +2668,7 @@
     <row r="3" ht="20" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Hydrocortisone</t>
+          <t>Dexamethasone</t>
         </is>
       </c>
       <c r="B3" s="2" t="n">
@@ -2681,16 +2681,16 @@
         <v>1</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>0.92</v>
+        <v>0.76</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>1.09</v>
+        <v>1.32</v>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Hydrocortisone + Fludrocortisone</t>
+          <t>Hydrocortisone</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -2703,16 +2703,16 @@
         <v>1</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>0.76</v>
+        <v>0.92</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>1.32</v>
+        <v>1.09</v>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Dexamethasone</t>
+          <t>Hydrocortisone + Fludrocortisone</t>
         </is>
       </c>
       <c r="B5" s="2" t="n">

</xml_diff>

<commit_message>
feat: sync latest NMA figure and table specification (v2026-09-21) with PRISMA dual-column standard, frequentist and Bayesian tracks, and reusable fill-in contracts
</commit_message>
<xml_diff>
--- a/examples/case_study_corticosteroids_nma/editable_files/office_docs/Master_Research_Database.xlsx
+++ b/examples/case_study_corticosteroids_nma/editable_files/office_docs/Master_Research_Database.xlsx
@@ -2646,7 +2646,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Methylprednisolone</t>
+          <t>Dexamethasone</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -2659,16 +2659,16 @@
         <v>1</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>0.82</v>
+        <v>0.76</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>1.22</v>
+        <v>1.32</v>
       </c>
     </row>
     <row r="3" ht="20" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Dexamethasone</t>
+          <t>Hydrocortisone + Fludrocortisone</t>
         </is>
       </c>
       <c r="B3" s="2" t="n">
@@ -2712,7 +2712,7 @@
     <row r="5" ht="20" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Hydrocortisone + Fludrocortisone</t>
+          <t>Methylprednisolone</t>
         </is>
       </c>
       <c r="B5" s="2" t="n">
@@ -2725,10 +2725,10 @@
         <v>1</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>0.76</v>
+        <v>0.82</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>1.32</v>
+        <v>1.22</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">

</xml_diff>

<commit_message>
feat: enforce resumable review formats and serial search checkpoints
</commit_message>
<xml_diff>
--- a/examples/case_study_corticosteroids_nma/editable_files/office_docs/Master_Research_Database.xlsx
+++ b/examples/case_study_corticosteroids_nma/editable_files/office_docs/Master_Research_Database.xlsx
@@ -8,8 +8,8 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Study_Characteristics" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Primary_Outcome_Mortality" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SUCRA_Rankings" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA_Primary_Outcome_Mortality" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA_Rankings_Not_Production_NMA" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2668,7 +2668,7 @@
     <row r="3" ht="20" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Hydrocortisone + Fludrocortisone</t>
+          <t>Methylprednisolone</t>
         </is>
       </c>
       <c r="B3" s="2" t="n">
@@ -2681,16 +2681,16 @@
         <v>1</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>0.76</v>
+        <v>0.82</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>1.32</v>
+        <v>1.22</v>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Hydrocortisone</t>
+          <t>Hydrocortisone + Fludrocortisone</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -2703,16 +2703,16 @@
         <v>1</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.76</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>1.09</v>
+        <v>1.32</v>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Methylprednisolone</t>
+          <t>Hydrocortisone</t>
         </is>
       </c>
       <c r="B5" s="2" t="n">
@@ -2725,10 +2725,10 @@
         <v>1</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>0.82</v>
+        <v>0.92</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>1.22</v>
+        <v>1.09</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">

</xml_diff>